<commit_message>
Scope the holding-vehicle rule to banking groups only
The vehicle-decides rule was applied to every holder, which was wrong in two
directions. It would have emptied the Insurance buckets, since most insurers
run an investment arm and would therefore have been reclassified as AMCs.
Worse, web research returned 'managed_funds' for Rawal Family Trust, which
under the old logic turned a private family trust into a Domestic AMC.

The rule now applies only where it was needed: 'Bank' is the one bucket with
no domestic/foreign split, so a banking group is classified by whether its
stake sits with the asset-management arm or on its own book. Every other
holder is classified by what the entity is.

Also flags medium-confidence entities for review, not just low, and records
Norges Bank under the new Foreign Pension Fund category since its holding is
reported as the Government Pension Fund Global. Foreign Government remains a
defensible alternative there, so it is flagged.
</commit_message>
<xml_diff>
--- a/output/ANANDRATHI_shareholder_categories.xlsx
+++ b/output/ANANDRATHI_shareholder_categories.xlsx
@@ -1049,6 +1049,11 @@
           <t>Azeez Family Trust</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Domestic corporate</t>
+        </is>
+      </c>
       <c r="D10" s="3" t="n">
         <v>4207494</v>
       </c>
@@ -1073,25 +1078,37 @@
         <v>3365054</v>
       </c>
       <c r="O10" s="3" t="n"/>
-      <c r="P10" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q10" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R10" s="4" t="n"/>
-      <c r="S10" s="4" t="n"/>
-      <c r="T10" s="4" t="n"/>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V10" s="4" t="n"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>private_family_trust</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>own_balance_sheet</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>https://trendlyne.com/equity/share-holding/747241/ANANDRATHI/31-03-2022/anand-rathi-wealth-ltd/</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1285,6 +1302,11 @@
           <t>Echjay Industries Pvt Ltd</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Domestic corporate</t>
+        </is>
+      </c>
       <c r="D14" s="3" t="n">
         <v>1683740</v>
       </c>
@@ -1309,25 +1331,37 @@
         <v>1675800</v>
       </c>
       <c r="O14" s="3" t="n"/>
-      <c r="P14" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q14" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R14" s="4" t="n"/>
-      <c r="S14" s="4" t="n"/>
-      <c r="T14" s="4" t="n"/>
-      <c r="U14" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V14" s="4" t="n"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>operating_company</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>operating_company_treasury</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>https://trendlyne.com/equity/share-holding/747241/ANANDRATHI/31-03-2022/anand-rathi-wealth-ltd/</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1767,6 +1801,11 @@
           <t>Norges Bank</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Foreign Pension Fund</t>
+        </is>
+      </c>
       <c r="D22" s="3" t="n">
         <v>897125</v>
       </c>
@@ -1793,23 +1832,39 @@
       <c r="O22" s="3" t="n"/>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>unresolved</t>
+          <t>web</t>
         </is>
       </c>
       <c r="Q22" s="4" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R22" s="4" t="n"/>
-      <c r="S22" s="4" t="n"/>
-      <c r="T22" s="4" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R22" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>pension_fund</t>
+        </is>
+      </c>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>pension_assets</t>
+        </is>
+      </c>
       <c r="U22" s="4" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="V22" s="4" t="n"/>
+      <c r="V22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.investing.com/equities/anand-rathi-wealth-ownership</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4387,6 +4442,11 @@
           <t>Nomura Holdings Inc</t>
         </is>
       </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
+        </is>
+      </c>
       <c r="D68" s="3" t="n"/>
       <c r="E68" s="3" t="n"/>
       <c r="F68" s="3" t="n"/>
@@ -4407,25 +4467,37 @@
         <v>9800</v>
       </c>
       <c r="O68" s="3" t="n"/>
-      <c r="P68" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q68" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R68" s="4" t="n"/>
-      <c r="S68" s="4" t="n"/>
-      <c r="T68" s="4" t="n"/>
-      <c r="U68" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V68" s="4" t="n"/>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>bank</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr"/>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Nomura_Holdings</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4436,6 +4508,11 @@
       <c r="B69" t="inlineStr">
         <is>
           <t>Nationwide Fund Advisors</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
         </is>
       </c>
       <c r="D69" s="3" t="n"/>
@@ -4454,25 +4531,37 @@
         <v>9682</v>
       </c>
       <c r="O69" s="3" t="n"/>
-      <c r="P69" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q69" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R69" s="4" t="n"/>
-      <c r="S69" s="4" t="n"/>
-      <c r="T69" s="4" t="n"/>
-      <c r="U69" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V69" s="4" t="n"/>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>asset_manager</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr"/>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>https://www.federalregister.gov/documents/2018/03/13/2018-05039/nationwide-fund-advisors-and-etf-series-solutions</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4899,6 +4988,11 @@
           <t>Angel One Ltd</t>
         </is>
       </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Domestic corporate</t>
+        </is>
+      </c>
       <c r="D77" s="3" t="n">
         <v>252</v>
       </c>
@@ -4925,23 +5019,39 @@
       <c r="O77" s="3" t="n"/>
       <c r="P77" s="4" t="inlineStr">
         <is>
-          <t>unresolved</t>
+          <t>web</t>
         </is>
       </c>
       <c r="Q77" s="4" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R77" s="4" t="n"/>
-      <c r="S77" s="4" t="n"/>
-      <c r="T77" s="4" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R77" s="4" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="S77" s="4" t="inlineStr">
+        <is>
+          <t>broker</t>
+        </is>
+      </c>
+      <c r="T77" s="4" t="inlineStr">
+        <is>
+          <t>custody_only</t>
+        </is>
+      </c>
       <c r="U77" s="4" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="V77" s="4" t="n"/>
+      <c r="V77" s="4" t="inlineStr">
+        <is>
+          <t>https://inc42.com/buzz/angel-one-amc-gets-sebi-nod-to-start-mutual-fund-business</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5008,6 +5118,11 @@
           <t>Legal &amp; General Group PLC</t>
         </is>
       </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Foreign Insurance</t>
+        </is>
+      </c>
       <c r="D79" s="3" t="n">
         <v>4328</v>
       </c>
@@ -5032,25 +5147,37 @@
         <v>4328</v>
       </c>
       <c r="O79" s="3" t="n"/>
-      <c r="P79" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q79" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R79" s="4" t="n"/>
-      <c r="S79" s="4" t="n"/>
-      <c r="T79" s="4" t="n"/>
-      <c r="U79" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V79" s="4" t="n"/>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>insurer</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr"/>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Legal_%26_General</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5061,6 +5188,11 @@
       <c r="B80" t="inlineStr">
         <is>
           <t>Franklin Templeton Inc</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
         </is>
       </c>
       <c r="D80" s="3" t="n"/>
@@ -5083,25 +5215,37 @@
         <v>3026</v>
       </c>
       <c r="O80" s="3" t="n"/>
-      <c r="P80" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q80" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R80" s="4" t="n"/>
-      <c r="S80" s="4" t="n"/>
-      <c r="T80" s="4" t="n"/>
-      <c r="U80" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V80" s="4" t="n"/>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>asset_manager</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr"/>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>https://www.ipqwery.com/ipowner/en/owner/ip/485181-franklin-resources-inc.html</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5166,6 +5310,11 @@
           <t>FlexShares Trust</t>
         </is>
       </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
+        </is>
+      </c>
       <c r="D82" s="3" t="n">
         <v>3072</v>
       </c>
@@ -5190,25 +5339,37 @@
         <v>1476</v>
       </c>
       <c r="O82" s="3" t="n"/>
-      <c r="P82" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q82" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R82" s="4" t="n"/>
-      <c r="S82" s="4" t="n"/>
-      <c r="T82" s="4" t="n"/>
-      <c r="U82" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V82" s="4" t="n"/>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>exchange_traded_fund_trust</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr"/>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>https://www.flexshares.com/us/en/individual/press</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5219,6 +5380,11 @@
       <c r="B83" t="inlineStr">
         <is>
           <t>Canadian Imperial Bank of Commerce</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
         </is>
       </c>
       <c r="D83" s="3" t="n"/>
@@ -5239,23 +5405,39 @@
       <c r="O83" s="3" t="n"/>
       <c r="P83" s="4" t="inlineStr">
         <is>
-          <t>unresolved</t>
+          <t>web</t>
         </is>
       </c>
       <c r="Q83" s="4" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R83" s="4" t="n"/>
-      <c r="S83" s="4" t="n"/>
-      <c r="T83" s="4" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R83" s="4" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="S83" s="4" t="inlineStr">
+        <is>
+          <t>bank</t>
+        </is>
+      </c>
+      <c r="T83" s="4" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
       <c r="U83" s="4" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="V83" s="4" t="n"/>
+      <c r="V83" s="4" t="inlineStr">
+        <is>
+          <t>https://www.marketscreener.com/quote/stock/CANADIAN-IMPERIAL-BANK-OF-40530896/company-shareholders</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5324,6 +5506,11 @@
       <c r="B85" t="inlineStr">
         <is>
           <t>Credit Agricole Group</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
         </is>
       </c>
       <c r="D85" s="3" t="n"/>
@@ -5344,25 +5531,37 @@
         <v>190</v>
       </c>
       <c r="O85" s="3" t="n"/>
-      <c r="P85" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q85" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R85" s="4" t="n"/>
-      <c r="S85" s="4" t="n"/>
-      <c r="T85" s="4" t="n"/>
-      <c r="U85" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V85" s="4" t="n"/>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>bank</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr"/>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>https://about.amundi.com/article/credit-agricole-sa-has-entered-exclusive-negotiations-societe-generale</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5373,6 +5572,11 @@
       <c r="B86" t="inlineStr">
         <is>
           <t>Deutsche Bank AG</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
         </is>
       </c>
       <c r="D86" s="3" t="n"/>
@@ -5397,25 +5601,37 @@
         <v>188</v>
       </c>
       <c r="O86" s="3" t="n"/>
-      <c r="P86" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q86" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R86" s="4" t="n"/>
-      <c r="S86" s="4" t="n"/>
-      <c r="T86" s="4" t="n"/>
-      <c r="U86" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V86" s="4" t="n"/>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>bank</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr"/>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/world/india/deutsche-banks-dws-buy-40-stake-nippon-life-india-asset-management-2025-11-13</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5475,6 +5691,11 @@
           <t>Prudential Financial Inc</t>
         </is>
       </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Foreign Insurance</t>
+        </is>
+      </c>
       <c r="D88" s="3" t="n"/>
       <c r="E88" s="3" t="n"/>
       <c r="F88" s="3" t="n">
@@ -5497,23 +5718,39 @@
       <c r="O88" s="3" t="n"/>
       <c r="P88" s="4" t="inlineStr">
         <is>
-          <t>unresolved</t>
+          <t>web</t>
         </is>
       </c>
       <c r="Q88" s="4" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R88" s="4" t="n"/>
-      <c r="S88" s="4" t="n"/>
-      <c r="T88" s="4" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R88" s="4" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="S88" s="4" t="inlineStr">
+        <is>
+          <t>insurer</t>
+        </is>
+      </c>
+      <c r="T88" s="4" t="inlineStr">
+        <is>
+          <t>insurance_float</t>
+        </is>
+      </c>
       <c r="U88" s="4" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="V88" s="4" t="n"/>
+      <c r="V88" s="4" t="inlineStr">
+        <is>
+          <t>https://ad-hoc-news.de/boerse/news/ueberblick/prudential-financial-balances-insuran/69743267</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5524,6 +5761,11 @@
       <c r="B89" t="inlineStr">
         <is>
           <t>FIL Ltd</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
         </is>
       </c>
       <c r="D89" s="3" t="n"/>
@@ -5540,25 +5782,37 @@
         <v>0</v>
       </c>
       <c r="O89" s="3" t="n"/>
-      <c r="P89" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q89" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R89" s="4" t="n"/>
-      <c r="S89" s="4" t="n"/>
-      <c r="T89" s="4" t="n"/>
-      <c r="U89" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V89" s="4" t="n"/>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>BM</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>asset_manager</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr"/>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Fidelity_International</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5569,6 +5823,11 @@
       <c r="B90" t="inlineStr">
         <is>
           <t>Russell Investments Group Ltd</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
         </is>
       </c>
       <c r="D90" s="3" t="n">
@@ -5595,23 +5854,39 @@
       <c r="O90" s="3" t="n"/>
       <c r="P90" s="4" t="inlineStr">
         <is>
-          <t>unresolved</t>
+          <t>web</t>
         </is>
       </c>
       <c r="Q90" s="4" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R90" s="4" t="n"/>
-      <c r="S90" s="4" t="n"/>
-      <c r="T90" s="4" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R90" s="4" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="S90" s="4" t="inlineStr">
+        <is>
+          <t>asset_manager</t>
+        </is>
+      </c>
+      <c r="T90" s="4" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
       <c r="U90" s="4" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="V90" s="4" t="n"/>
+      <c r="V90" s="4" t="inlineStr">
+        <is>
+          <t>https://find-and-update.company-information.service.gov.uk/company/12595999</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5942,6 +6217,11 @@
           <t>JPMorgan Chase &amp; Co</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
+        </is>
+      </c>
       <c r="D97" s="3" t="n"/>
       <c r="E97" s="3" t="n"/>
       <c r="F97" s="3" t="n">
@@ -5960,25 +6240,37 @@
         <v>0</v>
       </c>
       <c r="O97" s="3" t="n"/>
-      <c r="P97" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q97" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R97" s="4" t="n"/>
-      <c r="S97" s="4" t="n"/>
-      <c r="T97" s="4" t="n"/>
-      <c r="U97" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V97" s="4" t="n"/>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>bank</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr"/>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>https://jpmorganchaseco.gcs-web.com/static-files/3d1cfdc0-b391-4c71-a055-cb09f463622e</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5989,6 +6281,11 @@
       <c r="B98" t="inlineStr">
         <is>
           <t>Sun Life Financial Inc</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Foreign Insurance</t>
         </is>
       </c>
       <c r="D98" s="3" t="n"/>
@@ -6013,23 +6310,39 @@
       <c r="O98" s="3" t="n"/>
       <c r="P98" s="4" t="inlineStr">
         <is>
-          <t>unresolved</t>
+          <t>web</t>
         </is>
       </c>
       <c r="Q98" s="4" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R98" s="4" t="n"/>
-      <c r="S98" s="4" t="n"/>
-      <c r="T98" s="4" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R98" s="4" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="S98" s="4" t="inlineStr">
+        <is>
+          <t>insurer</t>
+        </is>
+      </c>
+      <c r="T98" s="4" t="inlineStr">
+        <is>
+          <t>insurance_float</t>
+        </is>
+      </c>
       <c r="U98" s="4" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="V98" s="4" t="n"/>
+      <c r="V98" s="4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Sun_Life_Financial</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6096,6 +6409,11 @@
           <t>Rawal Family Trust</t>
         </is>
       </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Domestic corporate</t>
+        </is>
+      </c>
       <c r="D100" s="3" t="n">
         <v>1750352</v>
       </c>
@@ -6116,25 +6434,37 @@
         <v>0</v>
       </c>
       <c r="O100" s="3" t="n"/>
-      <c r="P100" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q100" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R100" s="4" t="n"/>
-      <c r="S100" s="4" t="n"/>
-      <c r="T100" s="4" t="n"/>
-      <c r="U100" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V100" s="4" t="n"/>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>private_family_trust</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>own_balance_sheet</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr"/>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>https://trendlyne.com/equity/share-holding/747241/ANANDRATHI/31-03-2022/anand-rathi-wealth-ltd/</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6145,6 +6475,11 @@
       <c r="B101" t="inlineStr">
         <is>
           <t>SUHAS GUPTA FAMILY TRUST</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Domestic corporate</t>
         </is>
       </c>
       <c r="D101" s="3" t="n">
@@ -6171,25 +6506,37 @@
         <v>0</v>
       </c>
       <c r="O101" s="3" t="n"/>
-      <c r="P101" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q101" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R101" s="4" t="n"/>
-      <c r="S101" s="4" t="n"/>
-      <c r="T101" s="4" t="n"/>
-      <c r="U101" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V101" s="4" t="n"/>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>private_family_trust</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>own_balance_sheet</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr"/>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>https://trendlyne.com/equity/share-holding/747241/ANANDRATHI/31-03-2022/anand-rathi-wealth-ltd/</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6200,6 +6547,11 @@
       <c r="B102" t="inlineStr">
         <is>
           <t>Munix India Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Domestic corporate</t>
         </is>
       </c>
       <c r="D102" s="3" t="n">
@@ -6226,25 +6578,37 @@
         <v>0</v>
       </c>
       <c r="O102" s="3" t="n"/>
-      <c r="P102" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q102" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R102" s="4" t="n"/>
-      <c r="S102" s="4" t="n"/>
-      <c r="T102" s="4" t="n"/>
-      <c r="U102" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V102" s="4" t="n"/>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>operating_company</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>operating_company_treasury</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr"/>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>https://www.tofler.in/munix-india-private-limited/company/U00000PB2003PTC025986</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6255,6 +6619,11 @@
       <c r="B103" t="inlineStr">
         <is>
           <t>ANANDRATHI HOUSING FIN LTD</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Domestic corporate</t>
         </is>
       </c>
       <c r="D103" s="3" t="n">
@@ -6275,25 +6644,37 @@
         <v>0</v>
       </c>
       <c r="O103" s="3" t="n"/>
-      <c r="P103" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q103" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R103" s="4" t="n"/>
-      <c r="S103" s="4" t="n"/>
-      <c r="T103" s="4" t="n"/>
-      <c r="U103" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V103" s="4" t="n"/>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>operating_company</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>operating_company_treasury</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr"/>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>https://economictimes.indiatimes.com/company/anandrathi-housing-finance-limited/U67100MH2018PLC304174</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6304,6 +6685,11 @@
       <c r="B104" t="inlineStr">
         <is>
           <t>Wilshire Advisors LLC</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Foreign AMC</t>
         </is>
       </c>
       <c r="D104" s="3" t="n"/>
@@ -6320,25 +6706,37 @@
         <v>0</v>
       </c>
       <c r="O104" s="3" t="n"/>
-      <c r="P104" s="4" t="inlineStr">
-        <is>
-          <t>unresolved</t>
-        </is>
-      </c>
-      <c r="Q104" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="R104" s="4" t="n"/>
-      <c r="S104" s="4" t="n"/>
-      <c r="T104" s="4" t="n"/>
-      <c r="U104" s="4" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="V104" s="4" t="n"/>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>asset_manager</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>managed_funds</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr"/>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>https://www.wilshire.com</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>